<commit_message>
Publish EU IG version 0.0.2 with corrected dependency order
- Add new 0.0.2 release with hl7.terminology.r5 as first dependency
- Update version 0.0.1 to indicate it's superseded by 0.0.2
- Add 0.0.2 entries to package-feed.xml and publication-feed.xml
- Package-list.json now shows 0.0.2 as current version

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/docs/eu/StructureDefinition-ImComposition.xlsx
+++ b/docs/eu/StructureDefinition-ImComposition.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.0.1</t>
+    <t>0.0.2</t>
   </si>
   <si>
     <t>Name</t>
@@ -1497,7 +1497,7 @@
     <t>Composition.event:procedure.detail</t>
   </si>
   <si>
-    <t xml:space="preserve">CodeableReference(http://hl7.eu/fhir/imaging-r5/StructureDefinition/ImProcedure|0.0.1)
+    <t xml:space="preserve">CodeableReference(http://hl7.eu/fhir/imaging-r5/StructureDefinition/ImProcedure|0.0.2)
 </t>
   </si>
   <si>
@@ -1980,7 +1980,7 @@
     <t>Composition.section:procedure.entry:procedure</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(http://hl7.eu/fhir/imaging-r5/StructureDefinition/ImProcedure|0.0.1)
+    <t xml:space="preserve">Reference(http://hl7.eu/fhir/imaging-r5/StructureDefinition/ImProcedure|0.0.2)
 </t>
   </si>
   <si>
@@ -2111,7 +2111,7 @@
     <t>finding</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(http://hl7.eu/fhir/imaging-r5/StructureDefinition/ImFinding|0.0.1)
+    <t xml:space="preserve">Reference(http://hl7.eu/fhir/imaging-r5/StructureDefinition/ImFinding|0.0.2)
 </t>
   </si>
   <si>
@@ -2121,7 +2121,7 @@
     <t>keyimage</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(http://hl7.eu/fhir/imaging-r5/StructureDefinition/ImKeyImageDocumentReference|0.0.1|http://hl7.eu/fhir/imaging-r5/StructureDefinition/ImKeyImageImagingSelection|0.0.1)
+    <t xml:space="preserve">Reference(http://hl7.eu/fhir/imaging-r5/StructureDefinition/ImKeyImageDocumentReference|0.0.2|http://hl7.eu/fhir/imaging-r5/StructureDefinition/ImKeyImageImagingSelection|0.0.2)
 </t>
   </si>
   <si>

</xml_diff>